<commit_message>
feedback to -add the department
</commit_message>
<xml_diff>
--- a/Student_data.xlsx
+++ b/Student_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a28dfd3d4ea716f9/Desktop/Github_practice/github_practice/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3EEEEB1-C4F9-4DB0-B24F-10B47305B413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{B3EEEEB1-C4F9-4DB0-B24F-10B47305B413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4A172EB-293C-47A5-9BA7-18EF901647CB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FEC56B1F-0D84-4DEA-9D98-3A678254A11B}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Name</t>
   </si>
@@ -46,6 +46,12 @@
   </si>
   <si>
     <t>Python , Java, sql</t>
+  </si>
+  <si>
+    <t>Department</t>
+  </si>
+  <si>
+    <t>CSE</t>
   </si>
 </sst>
 </file>
@@ -397,8 +403,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B08B80AE-899B-4A2E-8787-33D1643A957E}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.5546875" customWidth="1"/>
+    <col min="2" max="2" width="17.109375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -414,6 +424,14 @@
       </c>
       <c r="B2" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>